<commit_message>
T-43: Correct Tiresias, who is not the Poet
Apply VarisPah's correction from issue 6 to the blockers note and the
Entities sheet of the public catalog. The Changes 2026-10-31 sheet keeps
the old name because it logs what changed that day.
</commit_message>
<xml_diff>
--- a/notes/Charon_Entity_Catalog_Public_2026-10-31.xlsx
+++ b/notes/Charon_Entity_Catalog_Public_2026-10-31.xlsx
@@ -6258,7 +6258,7 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>The Strategist. Arrives after cycle 6 at 25% chance. Wish is random from the 6 destinations. On arrival he meets Tiresias the Poet and the player chooses: Charybdis (lose 1 random memory, gain Moly) or Scylla (lose 1 random soul to a Wraith, Light -1, gain Nobody). The quest ends after the choice.</t>
+          <t>The Strategist. Arrives after cycle 6 at 25% chance. Wish is random from the 6 destinations. On arrival he meets Tiresias and the player chooses: Charybdis (lose 1 random memory, gain Moly) or Scylla (lose 1 random soul to a Wraith, Light -1, gain Nobody). The quest ends after the choice.</t>
         </is>
       </c>
     </row>
@@ -9688,7 +9688,7 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Tiresias the Poet</t>
+          <t>Tiresias</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -9703,7 +9703,7 @@
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>The named poet whom Odysseus meets before choosing a route.</t>
+          <t>The prophet whom Odysseus meets before choosing a route.</t>
         </is>
       </c>
       <c r="F84" s="3" t="inlineStr">
@@ -9733,7 +9733,7 @@
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>Named Tiresias the Poet. The quest text and soul table treat him as separate from the ordinary Poet soul.</t>
+          <t>Originally named Tiresias the Poet. Corrected Nov 1 (issue 6): he is not the Poet and appears only in the Odysseus encounter.</t>
         </is>
       </c>
     </row>

</xml_diff>